<commit_message>
data: publish 2026-09-20 sampler-linked operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-09-20-182路.xlsx
+++ b/data/export/2026-09-20-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC10"/>
+  <dimension ref="A1:AC18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -637,24 +637,24 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>07:13</t>
+          <t>07:16</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>68分钟</t>
+          <t>71分钟</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>06:21采样：该车到重点站唐陆公路龙东大道 ETA 15分钟；叠加该车自身同类时段从该站到终点历史中位数36分钟，约±5分钟</t>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -669,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -693,12 +693,12 @@
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>同车重点站剩余时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y2" s="2" t="inlineStr">
@@ -708,22 +708,22 @@
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA2" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
-          <t>68.0</t>
+          <t>72.0</t>
         </is>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>1/9</t>
+          <t>1/13</t>
         </is>
       </c>
     </row>
@@ -756,29 +756,29 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>07:19</t>
+          <t>07:25</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>70分钟</t>
+          <t>75分钟</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>06:21采样：该车到重点站博兴路东陆路 ETA 2分钟；叠加该车自身同类时段从该站到终点历史中位数56分钟，约±5分钟</t>
+          <t>SHMAAS多次终点ETA一致估算，约±4分钟</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -812,12 +812,12 @@
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
-          <t>同车重点站剩余时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y3" s="2" t="inlineStr">
@@ -837,12 +837,12 @@
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>75.0</t>
         </is>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>2/9</t>
+          <t>5/13</t>
         </is>
       </c>
     </row>
@@ -875,12 +875,12 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:32</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -892,12 +892,12 @@
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>06:21采样：该车到重点站新川路华东路 ETA 11分钟；叠加该车自身同类时段从该站到终点历史中位数59分钟，约±9分钟</t>
+          <t>SHMAAS多次终点ETA一致估算，约±4分钟</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -931,12 +931,12 @@
       </c>
       <c r="W4" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>同车重点站剩余时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y4" s="2" t="inlineStr">
@@ -946,12 +946,12 @@
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA4" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AB4" s="2" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>3/9</t>
+          <t>1/13</t>
         </is>
       </c>
     </row>
@@ -999,26 +999,22 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>07:47</t>
+          <t>07:54</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>72分钟</t>
+          <t>80分钟</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数72分钟估算，约±5分钟</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
+          <t>SHMAAS末次终点ETA推算：07:21采样，终点ETA 33分钟</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="inlineStr">
         <is>
           <t>06:01</t>
@@ -1026,7 +1022,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1050,12 +1046,12 @@
       </c>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>末次终点ETA兜底</t>
         </is>
       </c>
       <c r="Y5" s="2" t="inlineStr">
@@ -1065,22 +1061,22 @@
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA5" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
-          <t>72.0</t>
+          <t>75.5</t>
         </is>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>3/9</t>
+          <t>6/13</t>
         </is>
       </c>
     </row>
@@ -1113,29 +1109,29 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>07:51</t>
+          <t>07:53</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>76分钟</t>
+          <t>78分钟</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数76分钟估算，约±6分钟</t>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -1145,7 +1141,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1169,12 +1165,12 @@
       </c>
       <c r="W6" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X6" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y6" s="2" t="inlineStr">
@@ -1194,12 +1190,12 @@
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
-          <t>76.0</t>
+          <t>78.0</t>
         </is>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>7/9</t>
+          <t>9/13</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1260,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1303,12 +1299,12 @@
       </c>
       <c r="Z7" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA7" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AB7" s="2" t="inlineStr">
@@ -1318,7 +1314,7 @@
       </c>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>5/9</t>
+          <t>3/13</t>
         </is>
       </c>
     </row>
@@ -1326,24 +1322,24 @@
       <c r="A8" s="2" t="inlineStr"/>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>沪A32298D</t>
+          <t>沪A55712D</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>06:48</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
           <t>金杨路金口路</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>06:55</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>川沙客运站</t>
-        </is>
-      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -1356,34 +1352,34 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>08:15</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>80分钟</t>
+          <t>74分钟</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数80分钟估算，约±9分钟</t>
+          <t>07:21采样：该车到重点站唐陆公路锦绣东路 ETA 11分钟；叠加该车自身同类时段从该站到终点历史中位数29分钟，约±5分钟</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1397,7 +1393,7 @@
       <c r="T8" s="2" t="inlineStr"/>
       <c r="U8" s="2" t="inlineStr">
         <is>
-          <t>06:55</t>
+          <t>06:48</t>
         </is>
       </c>
       <c r="V8" s="2" t="inlineStr">
@@ -1412,7 +1408,7 @@
       </c>
       <c r="X8" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>同车重点站剩余时间</t>
         </is>
       </c>
       <c r="Y8" s="2" t="inlineStr">
@@ -1432,12 +1428,12 @@
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
-          <t>80.0</t>
+          <t>74.0</t>
         </is>
       </c>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>8/9</t>
+          <t>3/13</t>
         </is>
       </c>
     </row>
@@ -1445,24 +1441,24 @@
       <c r="A9" s="2" t="inlineStr"/>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>沪A12050A</t>
+          <t>沪A32298D</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>06:55</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
           <t>川沙客运站</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>07:00</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>金杨路金口路</t>
-        </is>
-      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -1475,30 +1471,34 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>08:15</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>81分钟</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr"/>
+          <t>07:21采样：该车到重点站东陆路金海路 ETA 5分钟；叠加该车自身同类时段从该站到终点历史中位数49分钟，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>06:01</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1512,7 +1512,7 @@
       <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>06:55</t>
         </is>
       </c>
       <c r="V9" s="2" t="inlineStr">
@@ -1522,17 +1522,17 @@
       </c>
       <c r="W9" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="X9" s="2" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>同车重点站剩余时间</t>
         </is>
       </c>
       <c r="Y9" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z9" s="2" t="inlineStr">
@@ -1542,13 +1542,17 @@
       </c>
       <c r="AA9" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB9" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB9" s="2" t="inlineStr">
+        <is>
+          <t>81.0</t>
+        </is>
+      </c>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>10/13</t>
         </is>
       </c>
     </row>
@@ -1556,24 +1560,24 @@
       <c r="A10" s="2" t="inlineStr"/>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>沪A68397D</t>
+          <t>沪A12050A</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
           <t>金杨路金口路</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>07:15</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>川沙客运站</t>
-        </is>
-      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -1586,34 +1590,30 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>08:28</t>
+          <t>待确认</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>74分钟</t>
+          <t>待确认</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数74分钟估算，约±7分钟</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>06:21</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1627,47 +1627,987 @@
       <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="inlineStr">
         <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="V10" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W10" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X10" s="2" t="inlineStr">
+        <is>
+          <t>证据不足</t>
+        </is>
+      </c>
+      <c r="Y10" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z10" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA10" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB10" s="2" t="inlineStr"/>
+      <c r="AC10" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>沪A35717D</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>08:26</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>74分钟</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数74分钟估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>06:11</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y11" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z11" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA11" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB11" s="2" t="inlineStr">
+        <is>
+          <t>74.0</t>
+        </is>
+      </c>
+      <c r="AC11" s="2" t="inlineStr">
+        <is>
+          <t>3/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>沪A68397D</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
           <t>07:15</t>
         </is>
       </c>
-      <c r="V10" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>08:31</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>76分钟</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>07:21采样：该车到重点站东陆路金海路 ETA 20分钟；叠加该车自身同类时段从该站到终点历史中位数49分钟，约±8分钟</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="V12" s="2" t="inlineStr">
         <is>
           <t>计划发车</t>
         </is>
       </c>
-      <c r="W10" s="2" t="inlineStr">
+      <c r="W12" s="2" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="X10" s="2" t="inlineStr">
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>同车重点站剩余时间</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z12" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA12" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB12" s="2" t="inlineStr">
+        <is>
+          <t>76.0</t>
+        </is>
+      </c>
+      <c r="AC12" s="2" t="inlineStr">
+        <is>
+          <t>7/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>沪A67026D</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>77分钟</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数77分钟估算，约±6分钟</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X13" s="2" t="inlineStr">
         <is>
           <t>同车历史全程时间</t>
         </is>
       </c>
-      <c r="Y10" s="2" t="inlineStr">
+      <c r="Y13" s="2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="Z10" s="2" t="inlineStr">
+      <c r="Z13" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA10" s="2" t="inlineStr">
+      <c r="AA13" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AB10" s="2" t="inlineStr">
-        <is>
-          <t>74.0</t>
-        </is>
-      </c>
-      <c r="AC10" s="2" t="inlineStr">
-        <is>
-          <t>5/9</t>
+      <c r="AB13" s="2" t="inlineStr">
+        <is>
+          <t>77.0</t>
+        </is>
+      </c>
+      <c r="AC13" s="2" t="inlineStr">
+        <is>
+          <t>8/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>沪A68870D</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>08:48</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>73分钟</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数73分钟估算，约±7分钟</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA14" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB14" s="2" t="inlineStr">
+        <is>
+          <t>72.0</t>
+        </is>
+      </c>
+      <c r="AC14" s="2" t="inlineStr">
+        <is>
+          <t>1/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>沪A67983D</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>08:57</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>81分钟</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数81分钟估算，约±9分钟</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB15" s="2" t="inlineStr">
+        <is>
+          <t>81.0</t>
+        </is>
+      </c>
+      <c r="AC15" s="2" t="inlineStr">
+        <is>
+          <t>10/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>沪A02126A</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="inlineStr"/>
+      <c r="T16" s="2" t="inlineStr"/>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W16" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X16" s="2" t="inlineStr">
+        <is>
+          <t>证据不足</t>
+        </is>
+      </c>
+      <c r="Y16" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z16" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA16" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB16" s="2" t="inlineStr"/>
+      <c r="AC16" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>沪A66513D</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>09:07</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>72分钟</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数72分钟估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr"/>
+      <c r="S17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="inlineStr"/>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X17" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z17" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA17" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB17" s="2" t="inlineStr">
+        <is>
+          <t>72.0</t>
+        </is>
+      </c>
+      <c r="AC17" s="2" t="inlineStr">
+        <is>
+          <t>1/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr"/>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>沪A31073D</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>09:26</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>71分钟</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数71分钟估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q18" s="2" t="inlineStr"/>
+      <c r="R18" s="2" t="inlineStr"/>
+      <c r="S18" s="2" t="inlineStr"/>
+      <c r="T18" s="2" t="inlineStr"/>
+      <c r="U18" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="V18" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W18" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X18" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y18" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z18" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA18" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB18" s="2" t="inlineStr">
+        <is>
+          <t>75.5</t>
+        </is>
+      </c>
+      <c r="AC18" s="2" t="inlineStr">
+        <is>
+          <t>6/13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: publish 2026-09-20 rolling operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-09-20-182路.xlsx
+++ b/data/export/2026-09-20-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC18"/>
+  <dimension ref="A1:AC23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -453,7 +453,7 @@
     <col width="14" customWidth="1" min="21" max="21"/>
     <col width="14" customWidth="1" min="22" max="22"/>
     <col width="12" customWidth="1" min="23" max="23"/>
-    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="22" customWidth="1" min="24" max="24"/>
     <col width="14" customWidth="1" min="25" max="25"/>
     <col width="18" customWidth="1" min="26" max="26"/>
     <col width="18" customWidth="1" min="27" max="27"/>
@@ -669,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -718,12 +718,12 @@
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
-          <t>72.0</t>
+          <t>75.5</t>
         </is>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>1/13</t>
+          <t>3/14</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -827,22 +827,22 @@
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA3" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
-          <t>75.0</t>
+          <t>73.5</t>
         </is>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>5/13</t>
+          <t>1/14</t>
         </is>
       </c>
     </row>
@@ -880,24 +880,24 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>07:32</t>
+          <t>07:33</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>72分钟</t>
+          <t>73分钟</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>SHMAAS多次终点ETA一致估算，约±4分钟</t>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -956,12 +956,12 @@
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
-          <t>72.0</t>
+          <t>74.0</t>
         </is>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>1/13</t>
+          <t>2/14</t>
         </is>
       </c>
     </row>
@@ -994,27 +994,31 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>07:54</t>
+          <t>08:02</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>80分钟</t>
+          <t>87分钟</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>SHMAAS末次终点ETA推算：07:21采样，终点ETA 33分钟</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr"/>
+          <t>SHMAAS终点近站ETA直接确认，约±2分钟</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
           <t>06:01</t>
@@ -1022,7 +1026,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1046,12 +1050,12 @@
       </c>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
-          <t>末次终点ETA兜底</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y5" s="2" t="inlineStr">
@@ -1071,12 +1075,12 @@
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
-          <t>75.5</t>
+          <t>79.0</t>
         </is>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>6/13</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -1114,24 +1118,24 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>07:53</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>78分钟</t>
+          <t>80分钟</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -1141,7 +1145,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1180,12 +1184,12 @@
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA6" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AB6" s="2" t="inlineStr">
@@ -1195,7 +1199,7 @@
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>9/13</t>
+          <t>4/14</t>
         </is>
       </c>
     </row>
@@ -1233,19 +1237,19 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>08:02</t>
+          <t>08:35</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>74分钟</t>
+          <t>107分钟</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数74分钟估算，约±5分钟</t>
+          <t>08:01采样：该车到重点站唐陆公路锦绣东路 ETA 2分钟；叠加该车自身同类时段从该站到终点历史中位数31分钟，约±5分钟</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -1260,7 +1264,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1289,7 +1293,7 @@
       </c>
       <c r="X7" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>同车重点站剩余时间</t>
         </is>
       </c>
       <c r="Y7" s="2" t="inlineStr">
@@ -1309,12 +1313,12 @@
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
-          <t>74.0</t>
+          <t>95.0</t>
         </is>
       </c>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>3/13</t>
+          <t>10/14</t>
         </is>
       </c>
     </row>
@@ -1347,29 +1351,29 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>08:01</t>
+          <t>08:08</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>74分钟</t>
+          <t>80分钟</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>07:21采样：该车到重点站唐陆公路锦绣东路 ETA 11分钟；叠加该车自身同类时段从该站到终点历史中位数29分钟，约±5分钟</t>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1379,7 +1383,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1403,12 +1407,12 @@
       </c>
       <c r="W8" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X8" s="2" t="inlineStr">
         <is>
-          <t>同车重点站剩余时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y8" s="2" t="inlineStr">
@@ -1418,22 +1422,22 @@
       </c>
       <c r="Z8" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA8" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
-          <t>74.0</t>
+          <t>79.0</t>
         </is>
       </c>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>3/13</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -1466,29 +1470,29 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>08:15</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>81分钟</t>
+          <t>84分钟</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>07:21采样：该车到重点站东陆路金海路 ETA 5分钟；叠加该车自身同类时段从该站到终点历史中位数49分钟，约±5分钟</t>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1498,7 +1502,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1522,12 +1526,12 @@
       </c>
       <c r="W9" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X9" s="2" t="inlineStr">
         <is>
-          <t>同车重点站剩余时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y9" s="2" t="inlineStr">
@@ -1547,12 +1551,12 @@
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
-          <t>81.0</t>
+          <t>84.0</t>
         </is>
       </c>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>10/13</t>
+          <t>8/14</t>
         </is>
       </c>
     </row>
@@ -1613,7 +1617,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1652,7 +1656,7 @@
       </c>
       <c r="Z10" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA10" s="2" t="inlineStr">
@@ -1663,7 +1667,7 @@
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr">
         <is>
-          <t>—/13</t>
+          <t>—/14</t>
         </is>
       </c>
     </row>
@@ -1701,19 +1705,19 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>08:26</t>
+          <t>08:35</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>74分钟</t>
+          <t>83分钟</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr"/>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数74分钟估算，约±5分钟</t>
+          <t>08:01采样：该车到重点站唐陆公路锦绣东路 ETA 2分钟；叠加该车自身同类时段从该站到终点历史中位数31分钟，约±5分钟</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
@@ -1728,7 +1732,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1757,7 +1761,7 @@
       </c>
       <c r="X11" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>同车重点站剩余时间</t>
         </is>
       </c>
       <c r="Y11" s="2" t="inlineStr">
@@ -1777,12 +1781,12 @@
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
-          <t>74.0</t>
+          <t>95.0</t>
         </is>
       </c>
       <c r="AC11" s="2" t="inlineStr">
         <is>
-          <t>3/13</t>
+          <t>10/14</t>
         </is>
       </c>
     </row>
@@ -1820,26 +1824,22 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>08:31</t>
+          <t>08:48</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>76分钟</t>
+          <t>94分钟</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>07:21采样：该车到重点站东陆路金海路 ETA 20分钟；叠加该车自身同类时段从该站到终点历史中位数49分钟，约±8分钟</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
+          <t>SHMAAS末次终点ETA推算：08:01采样，终点ETA 47分钟</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="inlineStr">
         <is>
           <t>06:01</t>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1871,17 +1871,17 @@
       </c>
       <c r="W12" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="X12" s="2" t="inlineStr">
         <is>
-          <t>同车重点站剩余时间</t>
+          <t>末次终点ETA兜底（误差可能&gt;15分钟）</t>
         </is>
       </c>
       <c r="Y12" s="2" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="Z12" s="2" t="inlineStr">
@@ -1891,17 +1891,13 @@
       </c>
       <c r="AA12" s="2" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AB12" s="2" t="inlineStr">
-        <is>
-          <t>76.0</t>
-        </is>
-      </c>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB12" s="2" t="inlineStr"/>
       <c r="AC12" s="2" t="inlineStr">
         <is>
-          <t>7/13</t>
+          <t>—/14</t>
         </is>
       </c>
     </row>
@@ -1939,24 +1935,24 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:48</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>77分钟</t>
+          <t>84分钟</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr"/>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数77分钟估算，约±6分钟</t>
+          <t>08:01采样：该车到重点站唐陆公路锦绣东路 ETA 11分钟；叠加该车自身同类时段从该站到终点历史中位数35分钟，约±5分钟</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
@@ -1966,7 +1962,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -1995,7 +1991,7 @@
       </c>
       <c r="X13" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>同车重点站剩余时间</t>
         </is>
       </c>
       <c r="Y13" s="2" t="inlineStr">
@@ -2015,12 +2011,12 @@
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
-          <t>77.0</t>
+          <t>84.0</t>
         </is>
       </c>
       <c r="AC13" s="2" t="inlineStr">
         <is>
-          <t>8/13</t>
+          <t>8/14</t>
         </is>
       </c>
     </row>
@@ -2058,24 +2054,24 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>08:48</t>
+          <t>08:55</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>73分钟</t>
+          <t>80分钟</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数73分钟估算，约±7分钟</t>
+          <t>08:01采样：该车到重点站唐陆公路春雅路 ETA 17分钟；叠加该车自身同类时段从该站到终点历史中位数36分钟，约±5分钟</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -2085,7 +2081,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -2114,7 +2110,7 @@
       </c>
       <c r="X14" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>同车重点站剩余时间</t>
         </is>
       </c>
       <c r="Y14" s="2" t="inlineStr">
@@ -2134,12 +2130,12 @@
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
-          <t>72.0</t>
+          <t>75.5</t>
         </is>
       </c>
       <c r="AC14" s="2" t="inlineStr">
         <is>
-          <t>1/13</t>
+          <t>3/14</t>
         </is>
       </c>
     </row>
@@ -2177,24 +2173,24 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>08:57</t>
+          <t>08:58</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>81分钟</t>
+          <t>82分钟</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数81分钟估算，约±9分钟</t>
+          <t>08:01采样：该车到重点站唐陆公路唐镇路 ETA 7分钟；叠加该车自身同类时段从该站到终点历史中位数49分钟，约±5分钟</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -2204,7 +2200,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -2233,7 +2229,7 @@
       </c>
       <c r="X15" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>同车重点站剩余时间</t>
         </is>
       </c>
       <c r="Y15" s="2" t="inlineStr">
@@ -2253,12 +2249,12 @@
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
-          <t>81.0</t>
+          <t>82.0</t>
         </is>
       </c>
       <c r="AC15" s="2" t="inlineStr">
         <is>
-          <t>10/13</t>
+          <t>7/14</t>
         </is>
       </c>
     </row>
@@ -2319,7 +2315,7 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -2369,7 +2365,7 @@
       <c r="AB16" s="2" t="inlineStr"/>
       <c r="AC16" s="2" t="inlineStr">
         <is>
-          <t>—/13</t>
+          <t>—/14</t>
         </is>
       </c>
     </row>
@@ -2407,24 +2403,24 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>09:07</t>
+          <t>09:09</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>72分钟</t>
+          <t>75分钟</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr"/>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数72分钟估算，约±5分钟</t>
+          <t>08:01采样：该车到重点站东陆路金海路 ETA 19分钟；叠加该车自身同类时段从该站到终点历史中位数49分钟，约±6分钟</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
@@ -2434,7 +2430,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -2463,7 +2459,7 @@
       </c>
       <c r="X17" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>同车重点站剩余时间</t>
         </is>
       </c>
       <c r="Y17" s="2" t="inlineStr">
@@ -2483,12 +2479,12 @@
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
-          <t>72.0</t>
+          <t>74.0</t>
         </is>
       </c>
       <c r="AC17" s="2" t="inlineStr">
         <is>
-          <t>1/13</t>
+          <t>2/14</t>
         </is>
       </c>
     </row>
@@ -2496,24 +2492,24 @@
       <c r="A18" s="2" t="inlineStr"/>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>沪A31073D</t>
+          <t>沪A13735A</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
           <t>金杨路金口路</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>08:15</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>川沙客运站</t>
-        </is>
-      </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -2526,19 +2522,19 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>09:26</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>71分钟</t>
+          <t>72分钟</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数71分钟估算，约±5分钟</t>
+          <t>08:01采样：该车到重点站新川路妙境路 ETA 8分钟；叠加该车自身同类时段从该站到终点历史中位数62分钟，约±5分钟</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
@@ -2553,7 +2549,7 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
@@ -2567,47 +2563,626 @@
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr">
         <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="V18" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W18" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X18" s="2" t="inlineStr">
+        <is>
+          <t>同车重点站剩余时间</t>
+        </is>
+      </c>
+      <c r="Y18" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z18" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA18" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB18" s="2" t="inlineStr">
+        <is>
+          <t>73.5</t>
+        </is>
+      </c>
+      <c r="AC18" s="2" t="inlineStr">
+        <is>
+          <t>1/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr"/>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>沪A31073D</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
           <t>08:15</t>
         </is>
       </c>
-      <c r="V18" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>09:26</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>71分钟</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数71分钟估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>08:01</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q19" s="2" t="inlineStr"/>
+      <c r="R19" s="2" t="inlineStr"/>
+      <c r="S19" s="2" t="inlineStr"/>
+      <c r="T19" s="2" t="inlineStr"/>
+      <c r="U19" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="V19" s="2" t="inlineStr">
         <is>
           <t>计划发车</t>
         </is>
       </c>
-      <c r="W18" s="2" t="inlineStr">
+      <c r="W19" s="2" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="X18" s="2" t="inlineStr">
+      <c r="X19" s="2" t="inlineStr">
         <is>
           <t>同车历史全程时间</t>
         </is>
       </c>
-      <c r="Y18" s="2" t="inlineStr">
+      <c r="Y19" s="2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="Z18" s="2" t="inlineStr">
+      <c r="Z19" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AA18" s="2" t="inlineStr">
+      <c r="AA19" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AB18" s="2" t="inlineStr">
-        <is>
-          <t>75.5</t>
-        </is>
-      </c>
-      <c r="AC18" s="2" t="inlineStr">
-        <is>
-          <t>6/13</t>
+      <c r="AB19" s="2" t="inlineStr">
+        <is>
+          <t>79.0</t>
+        </is>
+      </c>
+      <c r="AC19" s="2" t="inlineStr">
+        <is>
+          <t>5/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr"/>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>沪A67353D</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>09:31</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>76分钟</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数76分钟估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>08:01</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q20" s="2" t="inlineStr"/>
+      <c r="R20" s="2" t="inlineStr"/>
+      <c r="S20" s="2" t="inlineStr"/>
+      <c r="T20" s="2" t="inlineStr"/>
+      <c r="U20" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="V20" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W20" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X20" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y20" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z20" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA20" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB20" s="2" t="inlineStr">
+        <is>
+          <t>78.0</t>
+        </is>
+      </c>
+      <c r="AC20" s="2" t="inlineStr">
+        <is>
+          <t>4/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr"/>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>沪A08953A</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>08:31</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr"/>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>07:51</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>08:01</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q21" s="2" t="inlineStr"/>
+      <c r="R21" s="2" t="inlineStr"/>
+      <c r="S21" s="2" t="inlineStr"/>
+      <c r="T21" s="2" t="inlineStr"/>
+      <c r="U21" s="2" t="inlineStr">
+        <is>
+          <t>08:31</t>
+        </is>
+      </c>
+      <c r="V21" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W21" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X21" s="2" t="inlineStr">
+        <is>
+          <t>证据不足</t>
+        </is>
+      </c>
+      <c r="Y21" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z21" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA21" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB21" s="2" t="inlineStr"/>
+      <c r="AC21" s="2" t="inlineStr">
+        <is>
+          <t>—/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr"/>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>沪A55712D</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>08:35</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>09:53</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>78分钟</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数78分钟估算，约±8分钟</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>08:01</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q22" s="2" t="inlineStr"/>
+      <c r="R22" s="2" t="inlineStr"/>
+      <c r="S22" s="2" t="inlineStr"/>
+      <c r="T22" s="2" t="inlineStr"/>
+      <c r="U22" s="2" t="inlineStr">
+        <is>
+          <t>08:35</t>
+        </is>
+      </c>
+      <c r="V22" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W22" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X22" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y22" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z22" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA22" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB22" s="2" t="inlineStr">
+        <is>
+          <t>79.0</t>
+        </is>
+      </c>
+      <c r="AC22" s="2" t="inlineStr">
+        <is>
+          <t>5/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr"/>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>沪A12050A</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>08:55</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr"/>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>06:21</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>08:01</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q23" s="2" t="inlineStr"/>
+      <c r="R23" s="2" t="inlineStr"/>
+      <c r="S23" s="2" t="inlineStr"/>
+      <c r="T23" s="2" t="inlineStr"/>
+      <c r="U23" s="2" t="inlineStr">
+        <is>
+          <t>08:55</t>
+        </is>
+      </c>
+      <c r="V23" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W23" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X23" s="2" t="inlineStr">
+        <is>
+          <t>证据不足</t>
+        </is>
+      </c>
+      <c r="Y23" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z23" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA23" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB23" s="2" t="inlineStr"/>
+      <c r="AC23" s="2" t="inlineStr">
+        <is>
+          <t>—/14</t>
         </is>
       </c>
     </row>

</xml_diff>